<commit_message>
update smart recite mode
</commit_message>
<xml_diff>
--- a/LISTEN/Script/23_07_n3/23_07.xlsx
+++ b/LISTEN/Script/23_07_n3/23_07.xlsx
@@ -1609,7 +1609,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D31"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11.25" customWidth="1" min="1" max="1"/>
@@ -1641,6 +1641,11 @@
           <t>备注</t>
         </is>
       </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>History</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -1657,6 +1662,11 @@
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -1673,6 +1683,11 @@
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -1689,6 +1704,11 @@
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -1709,6 +1729,11 @@
           <t>幸福；幸运；好运</t>
         </is>
       </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -1725,6 +1750,11 @@
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -1741,6 +1771,11 @@
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -1757,6 +1792,7 @@
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -1777,6 +1813,7 @@
           <t>脱下；脱掉</t>
         </is>
       </c>
+      <c r="E9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -1793,6 +1830,7 @@
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -1809,6 +1847,7 @@
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -1829,6 +1868,7 @@
           <t>减少；降低；减轻</t>
         </is>
       </c>
+      <c r="E12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1845,6 +1885,7 @@
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1865,6 +1906,7 @@
           <t>近几年；这数年</t>
         </is>
       </c>
+      <c r="E14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1885,6 +1927,7 @@
           <t>攀登；登上</t>
         </is>
       </c>
+      <c r="E15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1905,6 +1948,7 @@
           <t>登山；爬山</t>
         </is>
       </c>
+      <c r="E16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1921,6 +1965,7 @@
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1937,6 +1982,7 @@
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1957,6 +2003,7 @@
           <t>出生；产生；出现</t>
         </is>
       </c>
+      <c r="E19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1973,6 +2020,7 @@
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1989,6 +2037,7 @@
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -2009,6 +2058,7 @@
           <t>赏花；观樱</t>
         </is>
       </c>
+      <c r="E22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -2025,6 +2075,7 @@
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -2041,6 +2092,7 @@
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -2057,6 +2109,7 @@
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -2073,6 +2126,7 @@
           <t>到来；来临</t>
         </is>
       </c>
+      <c r="E26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -2093,6 +2147,7 @@
           <t>走路方式</t>
         </is>
       </c>
+      <c r="E27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -2113,6 +2168,7 @@
           <t>上衣；外套</t>
         </is>
       </c>
+      <c r="E28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -2129,6 +2185,7 @@
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -2145,6 +2202,7 @@
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -2165,6 +2223,7 @@
           <t>后天</t>
         </is>
       </c>
+      <c r="E31" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>